<commit_message>
Update presentation and migration files for improved content
</commit_message>
<xml_diff>
--- a/arch/migracao_oci_aws.xlsx
+++ b/arch/migracao_oci_aws.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\clayton.oliveira\source\repos\files\arch\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2926C10-FFBC-4250-BF3A-5B684CFD06B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4655FBFB-BC49-47C7-9900-3AA590694A8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Custo - OCI" sheetId="5" r:id="rId1"/>
@@ -873,15 +873,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>71955</xdr:colOff>
       <xdr:row>13</xdr:row>
-      <xdr:rowOff>68888</xdr:rowOff>
+      <xdr:rowOff>158047</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>234995</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:colOff>321513</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>30766</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -911,8 +911,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="0" y="2450138"/>
-          <a:ext cx="10296570" cy="4388812"/>
+          <a:off x="71955" y="2551721"/>
+          <a:ext cx="10312928" cy="4428154"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1386,11 +1386,11 @@
         <v>0</v>
       </c>
       <c r="C8" s="6">
-        <v>4000</v>
+        <v>6000</v>
       </c>
       <c r="D8" s="7">
         <f t="shared" si="0"/>
-        <v>-4000</v>
+        <v>-6000</v>
       </c>
       <c r="E8" s="8">
         <f t="shared" si="1"/>
@@ -1432,15 +1432,15 @@
       </c>
       <c r="C10" s="12">
         <f t="shared" si="2"/>
-        <v>4800</v>
+        <v>6800</v>
       </c>
       <c r="D10" s="12">
         <f t="shared" si="2"/>
-        <v>29400</v>
+        <v>27400</v>
       </c>
       <c r="E10" s="13">
         <f t="shared" si="1"/>
-        <v>0.85964912280701755</v>
+        <v>0.80116959064327486</v>
       </c>
       <c r="F10" s="14"/>
     </row>
@@ -2269,15 +2269,15 @@
       </c>
       <c r="C53" s="18">
         <f t="shared" si="21"/>
-        <v>12540</v>
+        <v>14540</v>
       </c>
       <c r="D53" s="18">
         <f t="shared" si="21"/>
-        <v>36720</v>
+        <v>34720</v>
       </c>
       <c r="E53" s="19">
         <f>IF(B53=0,0,(B53-C53)/B53)</f>
-        <v>0.74543239951278928</v>
+        <v>0.7048315062931384</v>
       </c>
       <c r="F53" s="16"/>
     </row>
@@ -2307,7 +2307,7 @@
       </c>
       <c r="B57" s="20">
         <f>C53*12</f>
-        <v>150480</v>
+        <v>174480</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="B58" s="2">
         <f>D53*12</f>
-        <v>440640</v>
+        <v>416640</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -4655,7 +4655,7 @@
       </c>
       <c r="B19" s="2">
         <f>'Comparativo Mensal'!D53</f>
-        <v>36720</v>
+        <v>34720</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -4673,7 +4673,7 @@
       </c>
       <c r="B21" s="27">
         <f>IF(D16=0,0,(B19*12-D16)/D16)</f>
-        <v>7.4091603053435113</v>
+        <v>6.9511450381679385</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>

</xml_diff>